<commit_message>
Update momentum analysis scripts and add tight schedule results
</commit_message>
<xml_diff>
--- a/19:20/PLteamsData19:20_with_tight_schedule.xlsx
+++ b/19:20/PLteamsData19:20_with_tight_schedule.xlsx
@@ -1036,7 +1036,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1068,7 +1068,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1100,7 +1100,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1196,7 +1196,7 @@
         <v>6</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1228,7 +1228,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1292,7 +1292,7 @@
         <v>7</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1420,7 +1420,7 @@
         <v>5</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1452,7 +1452,7 @@
         <v>6</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1548,7 +1548,7 @@
         <v>5</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -1612,7 +1612,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1644,7 +1644,7 @@
         <v>5</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1708,7 +1708,7 @@
         <v>6</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1740,7 +1740,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1836,7 +1836,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1932,7 +1932,7 @@
         <v>7</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -2092,7 +2092,7 @@
         <v>6</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -2124,7 +2124,7 @@
         <v>6</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -2156,7 +2156,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2323,7 +2323,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -2867,7 +2867,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -2995,7 +2995,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -3027,7 +3027,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -3123,7 +3123,7 @@
         <v>6</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -3251,7 +3251,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -3347,7 +3347,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -3514,7 +3514,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -3546,7 +3546,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -3578,7 +3578,7 @@
         <v>6</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -3674,7 +3674,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -3706,7 +3706,7 @@
         <v>7</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -3866,7 +3866,7 @@
         <v>5</v>
       </c>
       <c r="J14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -3930,7 +3930,7 @@
         <v>7</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -4090,7 +4090,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -4122,7 +4122,7 @@
         <v>5</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -4186,7 +4186,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -4250,7 +4250,7 @@
         <v>6</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -4314,7 +4314,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -4346,7 +4346,7 @@
         <v>7</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -4474,7 +4474,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -4602,7 +4602,7 @@
         <v>6</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -4634,7 +4634,7 @@
         <v>6</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -4769,7 +4769,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4801,7 +4801,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -4929,7 +4929,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -4961,7 +4961,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -5025,7 +5025,7 @@
         <v>6</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -5057,7 +5057,7 @@
         <v>6</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -5089,7 +5089,7 @@
         <v>7</v>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -5153,7 +5153,7 @@
         <v>5</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -5185,7 +5185,7 @@
         <v>6</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -5249,7 +5249,7 @@
         <v>5</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -5345,7 +5345,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -5473,7 +5473,7 @@
         <v>5</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -5505,7 +5505,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -5729,7 +5729,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -5857,7 +5857,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -6024,7 +6024,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -6056,7 +6056,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -6088,7 +6088,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -6184,7 +6184,7 @@
         <v>6</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -6216,7 +6216,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -6280,7 +6280,7 @@
         <v>6</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -6408,7 +6408,7 @@
         <v>7</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -6568,7 +6568,7 @@
         <v>5</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -6600,7 +6600,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -6664,7 +6664,7 @@
         <v>6</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -6728,7 +6728,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -6792,7 +6792,7 @@
         <v>7</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -6888,7 +6888,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -6952,7 +6952,7 @@
         <v>5</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -6984,7 +6984,7 @@
         <v>5</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -7048,7 +7048,7 @@
         <v>6</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -7080,7 +7080,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -7112,7 +7112,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -7279,7 +7279,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -7311,7 +7311,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -7407,7 +7407,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -7439,7 +7439,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -7535,7 +7535,7 @@
         <v>5</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -7567,7 +7567,7 @@
         <v>7</v>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -7631,7 +7631,7 @@
         <v>5</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -7663,7 +7663,7 @@
         <v>7</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -7951,7 +7951,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -7983,7 +7983,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -8047,7 +8047,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -8079,7 +8079,7 @@
         <v>7</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -8143,7 +8143,7 @@
         <v>6</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -8303,7 +8303,7 @@
         <v>6</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -8335,7 +8335,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -8367,7 +8367,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -8534,7 +8534,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -8662,7 +8662,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -8694,7 +8694,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -9046,7 +9046,7 @@
         <v>5</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -9110,7 +9110,7 @@
         <v>6</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -9206,7 +9206,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -9238,7 +9238,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -9302,7 +9302,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -9334,7 +9334,7 @@
         <v>7</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -9398,7 +9398,7 @@
         <v>7</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -9462,7 +9462,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -9558,7 +9558,7 @@
         <v>6</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -9590,7 +9590,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -9622,7 +9622,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -9757,7 +9757,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -9789,7 +9789,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -9821,7 +9821,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -9949,7 +9949,7 @@
         <v>7</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -10013,7 +10013,7 @@
         <v>7</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -10109,7 +10109,7 @@
         <v>6</v>
       </c>
       <c r="J14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -10173,7 +10173,7 @@
         <v>7</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -10333,7 +10333,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -10397,7 +10397,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -10429,7 +10429,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -10461,7 +10461,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -10525,7 +10525,7 @@
         <v>6</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -10621,7 +10621,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -10685,7 +10685,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -10781,7 +10781,7 @@
         <v>6</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -10813,7 +10813,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -10845,7 +10845,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -11012,7 +11012,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -11044,7 +11044,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -11140,7 +11140,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -11172,7 +11172,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -11236,7 +11236,7 @@
         <v>6</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -11268,7 +11268,7 @@
         <v>7</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -11300,7 +11300,7 @@
         <v>6</v>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -11588,7 +11588,7 @@
         <v>7</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -11652,7 +11652,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -11716,7 +11716,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -11780,7 +11780,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -11812,7 +11812,7 @@
         <v>7</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -11876,7 +11876,7 @@
         <v>6</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -11940,7 +11940,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -12068,7 +12068,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -12267,7 +12267,7 @@
         <v>7</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -12299,7 +12299,7 @@
         <v>6</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -12395,7 +12395,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -12427,7 +12427,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -12459,7 +12459,7 @@
         <v>7</v>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -12587,7 +12587,7 @@
         <v>5</v>
       </c>
       <c r="J14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -12651,7 +12651,7 @@
         <v>6</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -12747,7 +12747,7 @@
         <v>6</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -12811,7 +12811,7 @@
         <v>5</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -12875,7 +12875,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -12907,7 +12907,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -12939,7 +12939,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -13003,7 +13003,7 @@
         <v>6</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -13035,7 +13035,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -13099,7 +13099,7 @@
         <v>6</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -13163,7 +13163,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -13259,7 +13259,7 @@
         <v>7</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -13490,7 +13490,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -13746,7 +13746,7 @@
         <v>5</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -14002,7 +14002,7 @@
         <v>6</v>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -14034,7 +14034,7 @@
         <v>5</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -14130,7 +14130,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -14162,7 +14162,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -14194,7 +14194,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -14258,7 +14258,7 @@
         <v>6</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -14290,7 +14290,7 @@
         <v>6</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -14354,7 +14354,7 @@
         <v>7</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -14418,7 +14418,7 @@
         <v>7</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -14482,7 +14482,7 @@
         <v>5</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -14514,7 +14514,7 @@
         <v>5</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -14713,7 +14713,7 @@
         <v>7</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -14745,7 +14745,7 @@
         <v>6</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -14841,7 +14841,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -14873,7 +14873,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -14937,7 +14937,7 @@
         <v>6</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -15257,7 +15257,7 @@
         <v>5</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -15289,7 +15289,7 @@
         <v>5</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -15353,7 +15353,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -15385,7 +15385,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -15481,7 +15481,7 @@
         <v>6</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -15513,7 +15513,7 @@
         <v>6</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -15641,7 +15641,7 @@
         <v>6</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -15737,7 +15737,7 @@
         <v>6</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -15769,7 +15769,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -15801,7 +15801,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -15936,7 +15936,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -15968,7 +15968,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -16000,7 +16000,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -16128,7 +16128,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -16224,7 +16224,7 @@
         <v>6</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -16256,7 +16256,7 @@
         <v>6</v>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -16384,7 +16384,7 @@
         <v>7</v>
       </c>
       <c r="J17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -16512,7 +16512,7 @@
         <v>5</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -16544,7 +16544,7 @@
         <v>6</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -16640,7 +16640,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -16672,7 +16672,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -16768,7 +16768,7 @@
         <v>6</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -16992,7 +16992,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -17024,7 +17024,7 @@
         <v>6</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -17056,7 +17056,7 @@
         <v>6</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -17191,7 +17191,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -17223,7 +17223,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -17255,7 +17255,7 @@
         <v>6</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -17351,7 +17351,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -17383,7 +17383,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -17575,7 +17575,7 @@
         <v>7</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -17639,7 +17639,7 @@
         <v>5</v>
       </c>
       <c r="J17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -17767,7 +17767,7 @@
         <v>7</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -17831,7 +17831,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -17895,7 +17895,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -17959,7 +17959,7 @@
         <v>5</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -18055,7 +18055,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -18119,7 +18119,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -18215,7 +18215,7 @@
         <v>7</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -18247,7 +18247,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -18279,7 +18279,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -18446,7 +18446,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -18478,7 +18478,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -18574,7 +18574,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -18606,7 +18606,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -18638,7 +18638,7 @@
         <v>7</v>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -18798,7 +18798,7 @@
         <v>7</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -18926,7 +18926,7 @@
         <v>5</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -18990,7 +18990,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -19054,7 +19054,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -19086,7 +19086,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -19118,7 +19118,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -19182,7 +19182,7 @@
         <v>7</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -19214,7 +19214,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -19342,7 +19342,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -19374,7 +19374,7 @@
         <v>5</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:10">
@@ -19470,7 +19470,7 @@
         <v>5</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -19502,7 +19502,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -19669,7 +19669,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -19829,7 +19829,7 @@
         <v>7</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -19893,7 +19893,7 @@
         <v>7</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -20053,7 +20053,7 @@
         <v>6</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -20277,7 +20277,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -20341,7 +20341,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -20405,7 +20405,7 @@
         <v>7</v>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -20437,7 +20437,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -20501,7 +20501,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -20565,7 +20565,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -20661,7 +20661,7 @@
         <v>7</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -20693,7 +20693,7 @@
         <v>7</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -20725,7 +20725,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -20860,7 +20860,7 @@
         <v>5</v>
       </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -20892,7 +20892,7 @@
         <v>5</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -20924,7 +20924,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -21020,7 +21020,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -21052,7 +21052,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -21116,7 +21116,7 @@
         <v>5</v>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -21244,7 +21244,7 @@
         <v>6</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -21500,7 +21500,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -21532,7 +21532,7 @@
         <v>6</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -21564,7 +21564,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -21660,7 +21660,7 @@
         <v>6</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -21724,7 +21724,7 @@
         <v>7</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -21788,7 +21788,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -21884,7 +21884,7 @@
         <v>7</v>
       </c>
       <c r="J35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:10">
@@ -22115,7 +22115,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -22147,7 +22147,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -22243,7 +22243,7 @@
         <v>6</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -22275,7 +22275,7 @@
         <v>5</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -22307,7 +22307,7 @@
         <v>7</v>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -22467,7 +22467,7 @@
         <v>5</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -22499,7 +22499,7 @@
         <v>5</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -22563,7 +22563,7 @@
         <v>5</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -22659,7 +22659,7 @@
         <v>6</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -22755,7 +22755,7 @@
         <v>6</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -22787,7 +22787,7 @@
         <v>7</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -22883,7 +22883,7 @@
         <v>6</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -22947,7 +22947,7 @@
         <v>6</v>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -23011,7 +23011,7 @@
         <v>7</v>
       </c>
       <c r="J32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -23139,7 +23139,7 @@
         <v>5</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -23171,7 +23171,7 @@
         <v>5</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -23338,7 +23338,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -23370,7 +23370,7 @@
         <v>7</v>
       </c>
       <c r="J5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -23466,7 +23466,7 @@
         <v>5</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -23498,7 +23498,7 @@
         <v>6</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -23530,7 +23530,7 @@
         <v>7</v>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -23594,7 +23594,7 @@
         <v>6</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -23626,7 +23626,7 @@
         <v>7</v>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -23722,7 +23722,7 @@
         <v>7</v>
       </c>
       <c r="J16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -23754,7 +23754,7 @@
         <v>5</v>
       </c>
       <c r="J17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -23914,7 +23914,7 @@
         <v>6</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -23978,7 +23978,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -24010,7 +24010,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -24106,7 +24106,7 @@
         <v>6</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -24138,7 +24138,7 @@
         <v>7</v>
       </c>
       <c r="J29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -24202,7 +24202,7 @@
         <v>6</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -24394,7 +24394,7 @@
         <v>6</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -24426,7 +24426,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -24593,7 +24593,7 @@
         <v>6</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -24753,7 +24753,7 @@
         <v>7</v>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -24849,7 +24849,7 @@
         <v>6</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -25073,7 +25073,7 @@
         <v>5</v>
       </c>
       <c r="J19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10">
@@ -25169,7 +25169,7 @@
         <v>7</v>
       </c>
       <c r="J22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -25233,7 +25233,7 @@
         <v>7</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -25265,7 +25265,7 @@
         <v>6</v>
       </c>
       <c r="J25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -25297,7 +25297,7 @@
         <v>7</v>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:10">
@@ -25361,7 +25361,7 @@
         <v>7</v>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -25457,7 +25457,7 @@
         <v>6</v>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -25617,7 +25617,7 @@
         <v>6</v>
       </c>
       <c r="J36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -25649,7 +25649,7 @@
         <v>7</v>
       </c>
       <c r="J37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -25681,7 +25681,7 @@
         <v>5</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:10">

</xml_diff>